<commit_message>
feat: Implement UI for registering new metric values with a dedicated drawer component and values page.
</commit_message>
<xml_diff>
--- a/data/database/metric_data.xlsx
+++ b/data/database/metric_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,29 @@
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>updated_at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Miguel Godoy</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>{"3": "Pangui", "4": "2026", "5": "1A"}</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-02-04 00:08:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Implement exportModal feature and button
</commit_message>
<xml_diff>
--- a/data/database/metric_data.xlsx
+++ b/data/database/metric_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,6 +475,75 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>2026-02-04 00:08:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Adolfo Farfal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{"3": "Pangui", "4": "2026", "5": "2A"}</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-02-04 00:10:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Claudio Beltrán</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>{"3": "Pullinque", "4": "2025", "5": "3A"}</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-02-04 00:10:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>{"Presidente":"Gabriel","Tesorero":"Felipe","Secretario":"Paulina","Inversión":"50000"}</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>{"4": "2026", "5": "1A"}</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-02-04 00:10:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add new template drawer component to manage template for ETL processes
</commit_message>
<xml_diff>
--- a/data/database/metric_data.xlsx
+++ b/data/database/metric_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,6 +454,11 @@
           <t>updated_at</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -477,6 +482,7 @@
           <t>2026-02-04 00:08:23</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -500,6 +506,7 @@
           <t>2026-02-04 00:10:05</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -523,6 +530,7 @@
           <t>2026-02-04 00:10:17</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -544,6 +552,31 @@
       <c r="E5" t="inlineStr">
         <is>
           <t>2026-02-04 00:10:54</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>{"Presidente": "Miguel", "Tesorero": "Andres", "Secretario": "Manuel", "Inversi\u00f3n": 100000}</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>{"4": "2026", "5": "2A"}</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-02-07T11:23:51.394515</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
reordenar: limpiar basura, mover tests fuera de la carpeta de libreria
</commit_message>
<xml_diff>
--- a/data/database/metric_data.xlsx
+++ b/data/database/metric_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,3047 +462,2567 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{"Presidente":"Gabriel","Tesorero":"Felipe","Secretario":"Paulina","Inversión":"50000"}</t>
+          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>{"4": "2026", "5": "1A"}</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-02-04 00:10:54</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>{"5": "2\u00b0 medio A", "6": "22992624-1", "7": "ALONSO JES\u00daS HERN\u00c1NDEZ AVENDA\u00d1O", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-02-13T11:51:15.122299</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{"Presidente": "Miguel", "Tesorero": "Andres", "Secretario": "Manuel", "Inversi\u00f3n": 100000}</t>
+          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>{"4": "2026", "5": "2A"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23075725-9", "7": "CARLOS ALBERTO NAVARRO NAHUEL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-07T11:23:51.394515</t>
+          <t>2026-02-13T11:51:15.123300</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Miguel Godoy</t>
+          <t>{"Buenas": 29, "Malas": 10, "Omitidas": 0, "Rend": 74.4, "SIMCE": 309, "Nota": 5.1, "Logro": "Adecuado", "Puntaje": 29}</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "1A", "6": "18720297-3"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23083703-1", "7": "DANTE FABI\u00c1N ULLOA MOLINA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-02-12T17:55:36.103828</t>
+          <t>2026-02-13T11:51:15.123300</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Jaime Jaimes</t>
+          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>{"3": "Panguipulli", "4": "2026", "5": "1A", "6": "12354-4"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23226019-K", "7": "ELMO ANDR\u00c9S MART\u00cdNEZ MERA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-02-12T17:55:36.103828</t>
+          <t>2026-02-13T11:51:15.123300</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Atila el Huno</t>
+          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "2A", "6": "2026-01-11 00:00:00"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "22305094-8", "7": "FABRICIANO ANTONIO CATAL\u00c1N HUEICHA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-02-12T17:55:36.103828</t>
+          <t>2026-02-13T11:51:15.123300</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Miguel Godoy</t>
+          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "1A", "6": "18720297-3"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23243196-2", "7": "FANNY LORETO COFR\u00c9 RIVAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-02-12T18:01:29.011630</t>
+          <t>2026-02-13T11:51:15.123300</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Jaime Jaimes</t>
+          <t>{"Buenas": 19, "Malas": 19, "Omitidas": 1, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>{"3": "Panguipulli", "4": "2026", "5": "1A", "6": "12354-4"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23264208-4", "7": "FELIPE ALFREDO BRAVO CONCHA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-02-12T18:01:29.011630</t>
+          <t>2026-02-13T11:51:15.123300</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Atila el Huno</t>
+          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "2A", "6": "2026-01-11 00:00:00"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23098425-5", "7": "FLORENCIA EMILIA HIRIART PULGAR", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-02-12T18:01:29.011630</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>12</v>
+        <v>32</v>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Miguel Godoy</t>
+          <t>{"Buenas": 28, "Malas": 11, "Omitidas": 0, "Rend": 71.8, "SIMCE": 303, "Nota": 4.9, "Logro": "Adecuado", "Puntaje": 28}</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "1A", "6": "18720297-3"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23311809-5", "7": "FRANCISCO ENRIQUE VILLARROEL FIGUEROA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-02-12T18:01:46.260527</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Jaime Jaimes</t>
+          <t>{"Buenas": 24, "Malas": 14, "Omitidas": 1, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>{"3": "Panguipulli", "4": "2026", "5": "1A", "6": "12354-4"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23142034-7", "7": "GABRIEL ARTURO CHEUQUEFILO NAUTULPAN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-02-12T18:01:46.260527</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Atila el Huno</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "2A", "6": "2026-01-11 00:00:00"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23283378-5", "7": "GUILLERMO ANDR\u00c9S SOLER CANIUCURA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-02-12T18:01:46.260527</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Miguel Godoy</t>
+          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "1A", "6": "18720297-3"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23190323-2", "7": "ISIDORA P\u00c9REZ OYARZ\u00daN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-02-12T18:01:59.834251</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Jaime Jaimes</t>
+          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>{"3": "Panguipulli", "4": "2026", "5": "1A", "6": "12354-4"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23254686-7", "7": "JAIME RUB\u00c9N VERA NEIHUAL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-02-12T18:01:59.834251</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Atila el Huno</t>
+          <t>{"Buenas": 18, "Malas": 20, "Omitidas": 1, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "2A", "6": "2026-01-11 00:00:00"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23303825-3", "7": "JOHANN FRANCISCO BENAVENTE JARAMILLO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-02-12T18:01:59.834251</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Miguel Godoy</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "1A", "6": "18720297-3"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23291819-5", "7": "JONATHAN F\u00c9LIX ACU\u00d1A MARIQUEO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-02-12T18:02:06.562947</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Jaime Jaimes</t>
+          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>{"3": "Panguipulli", "4": "2026", "5": "1A", "6": "12354-4"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "22747563-3", "7": "JOSSINH SIM\u00d3N VALDEBENITO RIVERA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-02-12T18:02:06.562947</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Atila el Huno</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "2A", "6": "2026-01-11 00:00:00"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23279870-K", "7": "LUCIANO ALBERTO DELGADO AYELEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-02-12T18:02:06.562947</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Miguel Godoy</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "1A", "6": "18720297-3"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23124964-8", "7": "PAOLO ELIAN CARRASCO GUAJARDO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-02-12T18:02:13.015581</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Jaime Jaimes</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>{"3": "Panguipulli", "4": "2026", "5": "1A", "6": "12354-4"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23335577-1", "7": "RICARDO JEREM\u00cdAS ANTONIO LICANCURA SALAZAR", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-02-12T18:02:13.015581</t>
+          <t>2026-02-13T11:51:15.124301</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Atila el Huno</t>
+          <t>{"Buenas": 32, "Malas": 7, "Omitidas": 0, "Rend": 82.1, "SIMCE": 326, "Nota": 5.7, "Logro": "Adecuado", "Puntaje": 32}</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>{"3": "Pullinque", "4": "2026", "5": "2A", "6": "2026-01-11 00:00:00"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23084146-2", "7": "SAMUEL ISMAEL INZUNZA CARTES", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-02-12T18:02:13.015581</t>
+          <t>2026-02-13T11:51:15.125804</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="B22" t="n">
         <v>4</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
+          <t>{"Buenas": 30, "Malas": 9, "Omitidas": 0, "Rend": 76.9, "SIMCE": 314, "Nota": 5.3, "Logro": "Adecuado", "Puntaje": 30}</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "22992624-1", "7": "ALONSO JES\u00daS HERN\u00c1NDEZ AVENDA\u00d1O", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23078776-K", "7": "VALENTINA IGNACIA VALENZUELA ESPARZA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.122299</t>
+          <t>2026-02-13T11:51:15.125804</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="B23" t="n">
         <v>4</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
+          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23075725-9", "7": "CARLOS ALBERTO NAVARRO NAHUEL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23165216-7", "7": "VALENTINA JAVIERA LLANQUIM\u00c1N ANTILLANCA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.123300</t>
+          <t>2026-02-13T11:51:15.125804</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B24" t="n">
         <v>4</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>{"Buenas": 29, "Malas": 10, "Omitidas": 0, "Rend": 74.4, "SIMCE": 309, "Nota": 5.1, "Logro": "Adecuado", "Puntaje": 29}</t>
+          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23083703-1", "7": "DANTE FABI\u00c1N ULLOA MOLINA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23178287-7", "7": "VICTORIA FLORENCIA CORT\u00c9S BETANCOURT", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.123300</t>
+          <t>2026-02-13T11:51:15.125804</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="B25" t="n">
         <v>4</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
+          <t>{"Buenas": 12, "Malas": 27, "Omitidas": 0, "Rend": 30.8, "SIMCE": 215, "Nota": 2.5, "Logro": "Insuficiente", "Puntaje": 12}</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23226019-K", "7": "ELMO ANDR\u00c9S MART\u00cdNEZ MERA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio A", "6": "23154617-0", "7": "YOAN PUNOY", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.123300</t>
+          <t>2026-02-13T11:51:15.125804</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="B26" t="n">
         <v>4</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
+          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "22305094-8", "7": "FABRICIANO ANTONIO CATAL\u00c1N HUEICHA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23092093-1", "7": "AARON ANTONIO RAIN MILLA\u00d1ANCO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.123300</t>
+          <t>2026-02-13T11:51:15.126808</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="B27" t="n">
         <v>4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
+          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23243196-2", "7": "FANNY LORETO COFR\u00c9 RIVAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23264494-K", "7": "ANAHI ANTONIA ESPARZA \u00c1LVAREZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.123300</t>
+          <t>2026-02-13T11:51:15.126808</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="B28" t="n">
         <v>4</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>{"Buenas": 19, "Malas": 19, "Omitidas": 1, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
+          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23264208-4", "7": "FELIPE ALFREDO BRAVO CONCHA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23332401-9", "7": "BEL\u00c9N JES\u00daS HUEITRA MATAMALA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.123300</t>
+          <t>2026-02-13T11:51:15.126808</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="B29" t="n">
         <v>4</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
+          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23098425-5", "7": "FLORENCIA EMILIA HIRIART PULGAR", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23307747-K", "7": "BENJAM\u00cdN EDUARDO ACU\u00d1A CURINAO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.126808</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="B30" t="n">
         <v>4</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>{"Buenas": 28, "Malas": 11, "Omitidas": 0, "Rend": 71.8, "SIMCE": 303, "Nota": 4.9, "Logro": "Adecuado", "Puntaje": 28}</t>
+          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23311809-5", "7": "FRANCISCO ENRIQUE VILLARROEL FIGUEROA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23248663-5", "7": "CAMILA ANTONIA PUNULAF QUISULEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127311</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="B31" t="n">
         <v>4</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>{"Buenas": 24, "Malas": 14, "Omitidas": 1, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
+          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23142034-7", "7": "GABRIEL ARTURO CHEUQUEFILO NAUTULPAN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23090987-3", "7": "CAMILO IGNACIO CASANOVA CONTRERAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127311</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="B32" t="n">
         <v>4</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23283378-5", "7": "GUILLERMO ANDR\u00c9S SOLER CANIUCURA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23096566-8", "7": "CARLOS MAT\u00cdAS PINILLA BRAVO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127823</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="B33" t="n">
         <v>4</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
+          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23190323-2", "7": "ISIDORA P\u00c9REZ OYARZ\u00daN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23136835-3", "7": "GIOHANS EDUARDO \u00d1ANCO HUILIP\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127823</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="B34" t="n">
         <v>4</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
+          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23254686-7", "7": "JAIME RUB\u00c9N VERA NEIHUAL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23307109-9", "7": "HENRY ARIEL KUTSCHER RAM\u00cdREZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127823</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="B35" t="n">
         <v>4</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>{"Buenas": 18, "Malas": 20, "Omitidas": 1, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
+          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23303825-3", "7": "JOHANN FRANCISCO BENAVENTE JARAMILLO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23129271-3", "7": "JAIME ALBERTO DELGADO MONCADA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127823</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="B36" t="n">
         <v>4</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23291819-5", "7": "JONATHAN F\u00c9LIX ACU\u00d1A MARIQUEO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23364347-5", "7": "JOAQU\u00cdN IGNACIO MU\u00d1OZ GU\u00cd\u00d1EZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127823</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="B37" t="n">
         <v>4</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
+          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "22747563-3", "7": "JOSSINH SIM\u00d3N VALDEBENITO RIVERA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23254876-2", "7": "JOAQU\u00cdN ISAAC VEL\u00c1SQUEZ WEVAR", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127823</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="B38" t="n">
         <v>4</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23279870-K", "7": "LUCIANO ALBERTO DELGADO AYELEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23170240-7", "7": "LUIS FELIPE SOBARZO MORALES", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127823</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="B39" t="n">
         <v>4</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 18, "Malas": 19, "Omitidas": 2, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23124964-8", "7": "PAOLO ELIAN CARRASCO GUAJARDO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23138672-6", "7": "MAGDALENA FRANSHESCA MU\u00d1OZ ALTAMIRANO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.127823</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="B40" t="n">
         <v>4</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23335577-1", "7": "RICARDO JEREM\u00cdAS ANTONIO LICANCURA SALAZAR", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23163042-2", "7": "MART\u00cdN ALEXIS CARIMAN CURI\u00d1ANCO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.124301</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="B41" t="n">
         <v>4</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>{"Buenas": 32, "Malas": 7, "Omitidas": 0, "Rend": 82.1, "SIMCE": 326, "Nota": 5.7, "Logro": "Adecuado", "Puntaje": 32}</t>
+          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23084146-2", "7": "SAMUEL ISMAEL INZUNZA CARTES", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "22583629-9", "7": "MART\u00cdN ALONSO CALDER\u00d3N MARILEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.125804</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="B42" t="n">
         <v>4</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>{"Buenas": 30, "Malas": 9, "Omitidas": 0, "Rend": 76.9, "SIMCE": 314, "Nota": 5.3, "Logro": "Adecuado", "Puntaje": 30}</t>
+          <t>{"Buenas": 29, "Malas": 10, "Omitidas": 0, "Rend": 74.4, "SIMCE": 309, "Nota": 5.1, "Logro": "Adecuado", "Puntaje": 29}</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23078776-K", "7": "VALENTINA IGNACIA VALENZUELA ESPARZA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23156392-K", "7": "MAT\u00cdAS CRISTOPHER OVANDO LEIVA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.125804</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="B43" t="n">
         <v>4</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
+          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23165216-7", "7": "VALENTINA JAVIERA LLANQUIM\u00c1N ANTILLANCA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23280628-1", "7": "MAXIMILIANO ANTONIO ARIAS SANDOVAL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.125804</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="B44" t="n">
         <v>4</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
+          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23178287-7", "7": "VICTORIA FLORENCIA CORT\u00c9S BETANCOURT", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23248366-0", "7": "NATACHA ANDREA PUNOI NAVARRETE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.125804</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="B45" t="n">
         <v>4</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>{"Buenas": 12, "Malas": 27, "Omitidas": 0, "Rend": 30.8, "SIMCE": 215, "Nota": 2.5, "Logro": "Insuficiente", "Puntaje": 12}</t>
+          <t>{"Buenas": 11, "Malas": 19, "Omitidas": 9, "Rend": 28.2, "SIMCE": 210, "Nota": 2.4, "Logro": "Insuficiente", "Puntaje": 11}</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio A", "6": "23154617-0", "7": "YOAN PUNOY", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23146205-8", "7": "PATRICIA MARIELA CATRILAF ANTIP\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.125804</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="B46" t="n">
         <v>4</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
+          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23092093-1", "7": "AARON ANTONIO RAIN MILLA\u00d1ANCO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23307151-K", "7": "VALERIE ARACELI HERRERA OLIVARES", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.126808</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="B47" t="n">
         <v>4</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
+          <t>{"Buenas": 15, "Malas": 24, "Omitidas": 0, "Rend": 38.5, "SIMCE": 232, "Nota": 2.9, "Logro": "Insuficiente", "Puntaje": 15}</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23264494-K", "7": "ANAHI ANTONIA ESPARZA \u00c1LVAREZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23356599-7", "7": "VICENTE ALEJANDRO AGUILERA CH\u00c1VEZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.126808</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="B48" t="n">
         <v>4</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
+          <t>{"Buenas": 31, "Malas": 8, "Omitidas": 0, "Rend": 79.5, "SIMCE": 320, "Nota": 5.5, "Logro": "Adecuado", "Puntaje": 31}</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23332401-9", "7": "BEL\u00c9N JES\u00daS HUEITRA MATAMALA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23126266-0", "7": "V\u00cdCTOR HUGO MAZA REINAHUEL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.126808</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="B49" t="n">
         <v>4</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
+          <t>{"Buenas": 12, "Malas": 27, "Omitidas": 0, "Rend": 30.8, "SIMCE": 215, "Nota": 2.5, "Logro": "Insuficiente", "Puntaje": 12}</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23307747-K", "7": "BENJAM\u00cdN EDUARDO ACU\u00d1A CURINAO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio B", "6": "23295647-K", "7": "YASMIN ANA\u00cdS AILLAP\u00c1N CATRILAF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.126808</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="B50" t="n">
         <v>4</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
+          <t>{"Buenas": 16, "Malas": 23, "Omitidas": 0, "Rend": 41.0, "SIMCE": 237, "Nota": 3.1, "Logro": "Insuficiente", "Puntaje": 16}</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23248663-5", "7": "CAMILA ANTONIA PUNULAF QUISULEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23096759-8", "7": "AIDETH ANAHIS ASTETE OBREQUE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127311</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="B51" t="n">
         <v>4</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23090987-3", "7": "CAMILO IGNACIO CASANOVA CONTRERAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23068616-5", "7": "ALONSO RAFAEL RODR\u00cdGUEZ AILLAP\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127311</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="B52" t="n">
         <v>4</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
+          <t>{"Buenas": 19, "Malas": 20, "Omitidas": 0, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23096566-8", "7": "CARLOS MAT\u00cdAS PINILLA BRAVO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23078035-8", "7": "ANGELICA ULLOA AGUAYO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127823</t>
+          <t>2026-02-13T11:51:15.128827</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="B53" t="n">
         <v>4</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
+          <t>{"Buenas": 19, "Malas": 20, "Omitidas": 0, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23136835-3", "7": "GIOHANS EDUARDO \u00d1ANCO HUILIP\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23367834-1", "7": "ANTONELLA ALEJANDRA CATRILAF RAIN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127823</t>
+          <t>2026-02-13T11:51:15.130329</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="B54" t="n">
         <v>4</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
+          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23307109-9", "7": "HENRY ARIEL KUTSCHER RAM\u00cdREZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23194865-1", "7": "ARACELLY DE LOS ANGELES CAYUFILO LEFIPAN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127823</t>
+          <t>2026-02-13T11:51:15.130329</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="B55" t="n">
         <v>4</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
+          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23129271-3", "7": "JAIME ALBERTO DELGADO MONCADA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23195825-8", "7": "BERNARDO AN\u00cdBAL RAINAHUEL CALLICUL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127823</t>
+          <t>2026-02-13T11:51:15.130329</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="B56" t="n">
         <v>4</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
+          <t>{"Buenas": 13, "Malas": 26, "Omitidas": 0, "Rend": 33.3, "SIMCE": 221, "Nota": 2.7, "Logro": "Insuficiente", "Puntaje": 13}</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23364347-5", "7": "JOAQU\u00cdN IGNACIO MU\u00d1OZ GU\u00cd\u00d1EZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23278997-2", "7": "DANIEL ALEXIS PE\u00d1A QUEUPUMIL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127823</t>
+          <t>2026-02-13T11:51:15.130329</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="B57" t="n">
         <v>4</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23254876-2", "7": "JOAQU\u00cdN ISAAC VEL\u00c1SQUEZ WEVAR", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23095273-6", "7": "DENISE ALINE CAMPOS BELTR\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127823</t>
+          <t>2026-02-13T11:51:15.131332</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="B58" t="n">
         <v>4</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23170240-7", "7": "LUIS FELIPE SOBARZO MORALES", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23266472-K", "7": "EMILIA VIANNEY ZARATE ROLD\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127823</t>
+          <t>2026-02-13T11:51:15.131332</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="B59" t="n">
         <v>4</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>{"Buenas": 18, "Malas": 19, "Omitidas": 2, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
+          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23138672-6", "7": "MAGDALENA FRANSHESCA MU\u00d1OZ ALTAMIRANO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23187256-6", "7": "ESPERANZA GALATAIA ANAHI CARTER CLAVIJO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.127823</t>
+          <t>2026-02-13T11:51:15.131332</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="B60" t="n">
         <v>4</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
+          <t>{"Buenas": 30, "Malas": 9, "Omitidas": 0, "Rend": 76.9, "SIMCE": 314, "Nota": 5.3, "Logro": "Adecuado", "Puntaje": 30}</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23163042-2", "7": "MART\u00cdN ALEXIS CARIMAN CURI\u00d1ANCO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23114253-3", "7": "FABI\u00c1N ESTEBAN ERICES REINUN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.131332</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="B61" t="n">
         <v>4</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
+          <t>{"Buenas": 24, "Malas": 14, "Omitidas": 1, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "22583629-9", "7": "MART\u00cdN ALONSO CALDER\u00d3N MARILEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23243775-8", "7": "FELIPE IGNACIO GODOY ROJAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.131332</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="B62" t="n">
         <v>4</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>{"Buenas": 29, "Malas": 10, "Omitidas": 0, "Rend": 74.4, "SIMCE": 309, "Nota": 5.1, "Logro": "Adecuado", "Puntaje": 29}</t>
+          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23156392-K", "7": "MAT\u00cdAS CRISTOPHER OVANDO LEIVA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23164005-3", "7": "FELIPE RICARDO CATRILEO PAILLALEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.131332</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="B63" t="n">
         <v>4</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
+          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23280628-1", "7": "MAXIMILIANO ANTONIO ARIAS SANDOVAL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23349462-3", "7": "FERNANDA VALESCA LUZ BRICE\u00d1O CALFUNAO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.131332</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="B64" t="n">
         <v>4</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
+          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23248366-0", "7": "NATACHA ANDREA PUNOI NAVARRETE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23015302-7", "7": "FRANCISCO ALEXANDER GARC\u00c9S RIVERA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.131332</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="B65" t="n">
         <v>4</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>{"Buenas": 11, "Malas": 19, "Omitidas": 9, "Rend": 28.2, "SIMCE": 210, "Nota": 2.4, "Logro": "Insuficiente", "Puntaje": 11}</t>
+          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23146205-8", "7": "PATRICIA MARIELA CATRILAF ANTIP\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23964755-3", "7": "FRANCO EZEQUIEL ZARATE ROLD\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.131332</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="B66" t="n">
         <v>4</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
+          <t>{"Buenas": 12, "Malas": 27, "Omitidas": 0, "Rend": 30.8, "SIMCE": 215, "Nota": 2.5, "Logro": "Insuficiente", "Puntaje": 12}</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23307151-K", "7": "VALERIE ARACELI HERRERA OLIVARES", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "22530419-K", "7": "GIOVANNY IGNACIO SAN MART\u00cdN PATI\u00d1O", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.132332</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="B67" t="n">
         <v>4</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>{"Buenas": 15, "Malas": 24, "Omitidas": 0, "Rend": 38.5, "SIMCE": 232, "Nota": 2.9, "Logro": "Insuficiente", "Puntaje": 15}</t>
+          <t>{"Buenas": 15, "Malas": 18, "Omitidas": 6, "Rend": 38.5, "SIMCE": 232, "Nota": 2.9, "Logro": "Insuficiente", "Puntaje": 15}</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23356599-7", "7": "VICENTE ALEJANDRO AGUILERA CH\u00c1VEZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23077073-5", "7": "H\u00c9CTOR ALEXIS VILLARROEL CONTRERAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.132332</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="B68" t="n">
         <v>4</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>{"Buenas": 31, "Malas": 8, "Omitidas": 0, "Rend": 79.5, "SIMCE": 320, "Nota": 5.5, "Logro": "Adecuado", "Puntaje": 31}</t>
+          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23126266-0", "7": "V\u00cdCTOR HUGO MAZA REINAHUEL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23195665-4", "7": "IGNACIO ALEJANDRO MONS\u00c1LVEZ RAM\u00d3N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.132332</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="B69" t="n">
         <v>4</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>{"Buenas": 12, "Malas": 27, "Omitidas": 0, "Rend": 30.8, "SIMCE": 215, "Nota": 2.5, "Logro": "Insuficiente", "Puntaje": 12}</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio B", "6": "23295647-K", "7": "YASMIN ANA\u00cdS AILLAP\u00c1N CATRILAF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23121281-7", "7": "JAVIERA JASM\u00cdN MARIFILO EPU\u00d1ANCO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.132332</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="B70" t="n">
         <v>4</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>{"Buenas": 16, "Malas": 23, "Omitidas": 0, "Rend": 41.0, "SIMCE": 237, "Nota": 3.1, "Logro": "Insuficiente", "Puntaje": 16}</t>
+          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23096759-8", "7": "AIDETH ANAHIS ASTETE OBREQUE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23237047-5", "7": "LUIS ALBERTO NAVARRETE COFR\u00c9", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.132332</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="B71" t="n">
         <v>4</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 5, "Malas": 28, "Omitidas": 6, "Rend": 12.8, "SIMCE": 177, "Nota": 1.6, "Logro": "Insuficiente", "Puntaje": 5}</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23068616-5", "7": "ALONSO RAFAEL RODR\u00cdGUEZ AILLAP\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23026868-1", "7": "LUIS MARIO LEFICHE HUICHULEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.132332</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="B72" t="n">
         <v>4</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>{"Buenas": 19, "Malas": 20, "Omitidas": 0, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
+          <t>{"Buenas": 21, "Malas": 17, "Omitidas": 1, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23078035-8", "7": "ANGELICA ULLOA AGUAYO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23003429-K", "7": "MARCELA ALEJANDRA CUR\u00cdN MONSALVE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.128827</t>
+          <t>2026-02-13T11:51:15.132332</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="B73" t="n">
         <v>4</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>{"Buenas": 19, "Malas": 20, "Omitidas": 0, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
+          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23367834-1", "7": "ANTONELLA ALEJANDRA CATRILAF RAIN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23225723-7", "7": "MARITZA ANDREA BELLO HUEITRA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.130329</t>
+          <t>2026-02-13T11:51:15.132332</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="B74" t="n">
         <v>4</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
+          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23194865-1", "7": "ARACELLY DE LOS ANGELES CAYUFILO LEFIPAN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23131840-2", "7": "MART\u00cdN FELIPE REINAHUEL MONTENEGRO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.130329</t>
+          <t>2026-02-13T11:51:15.133332</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="B75" t="n">
         <v>4</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
+          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23195825-8", "7": "BERNARDO AN\u00cdBAL RAINAHUEL CALLICUL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23076604-5", "7": "MARTINA ANTONELLA B\u00d3RQUEZ MU\u00d1OZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.130329</t>
+          <t>2026-02-13T11:51:15.133332</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="B76" t="n">
         <v>4</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>{"Buenas": 13, "Malas": 26, "Omitidas": 0, "Rend": 33.3, "SIMCE": 221, "Nota": 2.7, "Logro": "Insuficiente", "Puntaje": 13}</t>
+          <t>{"Buenas": 20, "Malas": 18, "Omitidas": 1, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23278997-2", "7": "DANIEL ALEXIS PE\u00d1A QUEUPUMIL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23276851-7", "7": "MARTINA ROC\u00cdO LE\u00d3N GONZ\u00c1LEZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.130329</t>
+          <t>2026-02-13T11:51:15.133332</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="B77" t="n">
         <v>4</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23095273-6", "7": "DENISE ALINE CAMPOS BELTR\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23138775-7", "7": "MAT\u00cdAS ANDR\u00c9S RAM\u00d3N MU\u00d1OZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.131332</t>
+          <t>2026-02-13T11:51:15.133332</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="B78" t="n">
         <v>4</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23266472-K", "7": "EMILIA VIANNEY ZARATE ROLD\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "20338382-7", "7": "MAXIMO RAIMUNDO PA\u00d1IAN JARAMILLO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.131332</t>
+          <t>2026-02-13T11:51:15.133332</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="B79" t="n">
         <v>4</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
+          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23187256-6", "7": "ESPERANZA GALATAIA ANAHI CARTER CLAVIJO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23366739-0", "7": "MELIXA ALEJANDRA LEFINAO LLANCAP\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.131332</t>
+          <t>2026-02-13T11:51:15.133332</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>82</v>
+        <v>102</v>
       </c>
       <c r="B80" t="n">
         <v>4</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>{"Buenas": 30, "Malas": 9, "Omitidas": 0, "Rend": 76.9, "SIMCE": 314, "Nota": 5.3, "Logro": "Adecuado", "Puntaje": 30}</t>
+          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23114253-3", "7": "FABI\u00c1N ESTEBAN ERICES REINUN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23298489-9", "7": "RENATO FRANCISCO CANIULEF CATRICURA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.131332</t>
+          <t>2026-02-13T11:51:15.133332</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="B81" t="n">
         <v>4</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>{"Buenas": 24, "Malas": 14, "Omitidas": 1, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
+          <t>{"Buenas": 19, "Malas": 20, "Omitidas": 0, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23243775-8", "7": "FELIPE IGNACIO GODOY ROJAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23332611-9", "7": "RICARDO ARTURO CHOCORI CHOCORI", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.131332</t>
+          <t>2026-02-13T11:51:15.133332</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="B82" t="n">
         <v>4</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
+          <t>{"Buenas": 17, "Malas": 22, "Omitidas": 0, "Rend": 43.6, "SIMCE": 243, "Nota": 3.2, "Logro": "Elemental", "Puntaje": 17}</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23164005-3", "7": "FELIPE RICARDO CATRILEO PAILLALEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio C", "6": "23203396-7", "7": "SEBASTIAN MILLACURA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.131332</t>
+          <t>2026-02-13T11:51:15.133332</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="B83" t="n">
         <v>4</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
+          <t>{"Buenas": 10, "Malas": 28, "Omitidas": 1, "Rend": 25.6, "SIMCE": 204, "Nota": 2.3, "Logro": "Insuficiente", "Puntaje": 10}</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23349462-3", "7": "FERNANDA VALESCA LUZ BRICE\u00d1O CALFUNAO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23260659-2", "7": "BENJAM\u00cdN ALONSO RUIZ SEP\u00daLVEDA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.131332</t>
+          <t>2026-02-13T11:51:15.134332</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>86</v>
+        <v>106</v>
       </c>
       <c r="B84" t="n">
         <v>4</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
+          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23015302-7", "7": "FRANCISCO ALEXANDER GARC\u00c9S RIVERA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23147648-2", "7": "CONSTANZA MAGDALENA HERN\u00c1NDEZ PARADA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.131332</t>
+          <t>2026-02-13T11:51:15.134332</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="B85" t="n">
         <v>4</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
+          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23964755-3", "7": "FRANCO EZEQUIEL ZARATE ROLD\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23123655-4", "7": "DANIEL ALEJANDRO ARANEDA INFANTE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.131332</t>
+          <t>2026-02-13T11:51:15.134332</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>88</v>
+        <v>108</v>
       </c>
       <c r="B86" t="n">
         <v>4</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>{"Buenas": 12, "Malas": 27, "Omitidas": 0, "Rend": 30.8, "SIMCE": 215, "Nota": 2.5, "Logro": "Insuficiente", "Puntaje": 12}</t>
+          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "22530419-K", "7": "GIOVANNY IGNACIO SAN MART\u00cdN PATI\u00d1O", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "22623080-7", "7": "ELISA N\u00d6EL CASTILLO PASTENE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.132332</t>
+          <t>2026-02-13T11:51:15.134332</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>89</v>
+        <v>109</v>
       </c>
       <c r="B87" t="n">
         <v>4</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>{"Buenas": 15, "Malas": 18, "Omitidas": 6, "Rend": 38.5, "SIMCE": 232, "Nota": 2.9, "Logro": "Insuficiente", "Puntaje": 15}</t>
+          <t>{"Buenas": 16, "Malas": 23, "Omitidas": 0, "Rend": 41.0, "SIMCE": 237, "Nota": 3.1, "Logro": "Insuficiente", "Puntaje": 16}</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23077073-5", "7": "H\u00c9CTOR ALEXIS VILLARROEL CONTRERAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23222221-2", "7": "FABI\u00c1N ESTEBAN ALIU LINCOCHEO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.132332</t>
+          <t>2026-02-13T11:51:15.134332</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="B88" t="n">
         <v>4</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
+          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23195665-4", "7": "IGNACIO ALEJANDRO MONS\u00c1LVEZ RAM\u00d3N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23223725-2", "7": "FELIPE EUGENIO CARIP\u00c1N LLAPELEO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.132332</t>
+          <t>2026-02-13T11:51:15.134332</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>91</v>
+        <v>111</v>
       </c>
       <c r="B89" t="n">
         <v>4</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23121281-7", "7": "JAVIERA JASM\u00cdN MARIFILO EPU\u00d1ANCO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23209728-0", "7": "FELIPE IGNACIO LARA CAMPOS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.132332</t>
+          <t>2026-02-13T11:51:15.134332</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="B90" t="n">
         <v>4</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>{"Buenas": 18, "Malas": 21, "Omitidas": 0, "Rend": 46.2, "SIMCE": 248, "Nota": 3.3, "Logro": "Elemental", "Puntaje": 18}</t>
+          <t>{"Buenas": 28, "Malas": 11, "Omitidas": 0, "Rend": 71.8, "SIMCE": 303, "Nota": 4.9, "Logro": "Adecuado", "Puntaje": 28}</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23237047-5", "7": "LUIS ALBERTO NAVARRETE COFR\u00c9", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23075733-K", "7": "FRANKO JUSTINO CARRASCO BETANCOURT", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.132332</t>
+          <t>2026-02-13T11:51:15.134332</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>93</v>
+        <v>113</v>
       </c>
       <c r="B91" t="n">
         <v>4</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>{"Buenas": 5, "Malas": 28, "Omitidas": 6, "Rend": 12.8, "SIMCE": 177, "Nota": 1.6, "Logro": "Insuficiente", "Puntaje": 5}</t>
+          <t>{"Buenas": 12, "Malas": 27, "Omitidas": 0, "Rend": 30.8, "SIMCE": 215, "Nota": 2.5, "Logro": "Insuficiente", "Puntaje": 12}</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23026868-1", "7": "LUIS MARIO LEFICHE HUICHULEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "22600443-2", "7": "GUSTAVO JES\u00daS GUAJARDO LLONCO\u00d1ANCO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.132332</t>
+          <t>2026-02-13T11:51:15.135332</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>94</v>
+        <v>114</v>
       </c>
       <c r="B92" t="n">
         <v>4</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>{"Buenas": 21, "Malas": 17, "Omitidas": 1, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
+          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23003429-K", "7": "MARCELA ALEJANDRA CUR\u00cdN MONSALVE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23206392-0", "7": "HORTENCIA ALEJANDRA ANCAMILLA MILLAL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.132332</t>
+          <t>2026-02-13T11:51:15.135332</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="B93" t="n">
         <v>4</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
+          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23225723-7", "7": "MARITZA ANDREA BELLO HUEITRA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23071865-2", "7": "ISMAEL LUCIANO CALFI\u00d1IR HUENU\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.132332</t>
+          <t>2026-02-13T11:51:15.135332</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="B94" t="n">
         <v>4</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
+          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23131840-2", "7": "MART\u00cdN FELIPE REINAHUEL MONTENEGRO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23284555-4", "7": "JAVIER IGNACIO OLAVARR\u00cdA CUEVAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.133332</t>
+          <t>2026-02-13T11:51:15.135332</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>97</v>
+        <v>117</v>
       </c>
       <c r="B95" t="n">
         <v>4</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
+          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23076604-5", "7": "MARTINA ANTONELLA B\u00d3RQUEZ MU\u00d1OZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "24309656-1", "7": "JEANEN PE\u00d1A", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.133332</t>
+          <t>2026-02-13T11:51:15.135332</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>98</v>
+        <v>118</v>
       </c>
       <c r="B96" t="n">
         <v>4</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>{"Buenas": 20, "Malas": 18, "Omitidas": 1, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
+          <t>{"Buenas": 27, "Malas": 11, "Omitidas": 1, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23276851-7", "7": "MARTINA ROC\u00cdO LE\u00d3N GONZ\u00c1LEZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23210749-9", "7": "LILIANA IGNACIA MADARIAGA ANCAMILLA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.133332</t>
+          <t>2026-02-13T11:51:15.136332</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="B97" t="n">
         <v>4</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
+          <t>{"Buenas": 19, "Malas": 20, "Omitidas": 0, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23138775-7", "7": "MAT\u00cdAS ANDR\u00c9S RAM\u00d3N MU\u00d1OZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23201622-1", "7": "LUCAS IGNACIO BENJAM\u00cdN ALA\u00d1ANCO BRICE\u00d1O", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.133332</t>
+          <t>2026-02-13T11:51:15.136332</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="B98" t="n">
         <v>4</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
+          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "20338382-7", "7": "MAXIMO RAIMUNDO PA\u00d1IAN JARAMILLO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23169236-3", "7": "MADELEINE INES P\u00c9REZ ESPINOZA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.133332</t>
+          <t>2026-02-13T11:51:15.136332</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>101</v>
+        <v>121</v>
       </c>
       <c r="B99" t="n">
         <v>4</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
+          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23366739-0", "7": "MELIXA ALEJANDRA LEFINAO LLANCAP\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "22596306-1", "7": "MARTINA ANA\u00cdS G\u00d3MEZ PACHECO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.133332</t>
+          <t>2026-02-13T11:51:15.136332</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="B100" t="n">
         <v>4</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>{"Buenas": 25, "Malas": 14, "Omitidas": 0, "Rend": 64.1, "SIMCE": 287, "Nota": 4.3, "Logro": "Elemental", "Puntaje": 25}</t>
+          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23298489-9", "7": "RENATO FRANCISCO CANIULEF CATRICURA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23221210-1", "7": "MARTINA PASCAL LEFIQUEO ANTILEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.133332</t>
+          <t>2026-02-13T11:51:15.136332</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>103</v>
+        <v>123</v>
       </c>
       <c r="B101" t="n">
         <v>4</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>{"Buenas": 19, "Malas": 20, "Omitidas": 0, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
+          <t>{"Buenas": 13, "Malas": 26, "Omitidas": 0, "Rend": 33.3, "SIMCE": 221, "Nota": 2.7, "Logro": "Insuficiente", "Puntaje": 13}</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23332611-9", "7": "RICARDO ARTURO CHOCORI CHOCORI", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23207278-4", "7": "MAT\u00cdAS FRANCHESCO \u00c1LAMOS LLEUFUMAN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.133332</t>
+          <t>2026-02-13T11:51:15.136332</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="B102" t="n">
         <v>4</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>{"Buenas": 17, "Malas": 22, "Omitidas": 0, "Rend": 43.6, "SIMCE": 243, "Nota": 3.2, "Logro": "Elemental", "Puntaje": 17}</t>
+          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio C", "6": "23203396-7", "7": "SEBASTIAN MILLACURA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23020358-K", "7": "MOIS\u00c9S ALONSO DUR\u00c1N BERROCAL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.133332</t>
+          <t>2026-02-13T11:51:15.137331</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="B103" t="n">
         <v>4</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>{"Buenas": 10, "Malas": 28, "Omitidas": 1, "Rend": 25.6, "SIMCE": 204, "Nota": 2.3, "Logro": "Insuficiente", "Puntaje": 10}</t>
+          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23260659-2", "7": "BENJAM\u00cdN ALONSO RUIZ SEP\u00daLVEDA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "22833690-4", "7": "NAYELI MANQUELIPE BURGOS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.134332</t>
+          <t>2026-02-13T11:51:15.137331</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="B104" t="n">
         <v>4</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
+          <t>{"Buenas": 29, "Malas": 10, "Omitidas": 0, "Rend": 74.4, "SIMCE": 309, "Nota": 5.1, "Logro": "Adecuado", "Puntaje": 29}</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23147648-2", "7": "CONSTANZA MAGDALENA HERN\u00c1NDEZ PARADA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23177773-3", "7": "NEYBER BENJAM\u00cdN CHAND\u00cdA MERA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.134332</t>
+          <t>2026-02-13T11:51:15.137331</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="B105" t="n">
         <v>4</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
+          <t>{"Buenas": 16, "Malas": 23, "Omitidas": 0, "Rend": 41.0, "SIMCE": 237, "Nota": 3.1, "Logro": "Insuficiente", "Puntaje": 16}</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23123655-4", "7": "DANIEL ALEJANDRO ARANEDA INFANTE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23061855-0", "7": "RODRIGO FERNANDO CH\u00c1VEZ MONS\u00c1LVEZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.134332</t>
+          <t>2026-02-13T11:51:15.137331</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="B106" t="n">
         <v>4</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
+          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio D", "6": "22623080-7", "7": "ELISA N\u00d6EL CASTILLO PASTENE", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23229067-6", "7": "SIGRID NAYARETH BEL\u00c9N BURGOS ESPINOZA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.134332</t>
+          <t>2026-02-13T11:51:15.137834</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>109</v>
+        <v>129</v>
       </c>
       <c r="B107" t="n">
         <v>4</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>{"Buenas": 16, "Malas": 23, "Omitidas": 0, "Rend": 41.0, "SIMCE": 237, "Nota": 3.1, "Logro": "Insuficiente", "Puntaje": 16}</t>
+          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23222221-2", "7": "FABI\u00c1N ESTEBAN ALIU LINCOCHEO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23296820-6", "7": "TERECITA DEL NI\u00d1O JES\u00daS CARES MONS\u00c1LVEZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-02-13T11:51:15.134332</t>
+          <t>2026-02-13T11:51:15.137834</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="B108" t="n">
         <v>4</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
+          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23223725-2", "7": "FELIPE EUGENIO CARIP\u00c1N LLAPELEO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
+          <t>{"5": "2\u00b0 medio D", "6": "23077160-K", "7": "YOHAN RICARDO PROVOTH ARAVENA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.134332</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
-        <v>111</v>
-      </c>
-      <c r="B109" t="n">
-        <v>4</v>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>{"Buenas": 14, "Malas": 25, "Omitidas": 0, "Rend": 35.9, "SIMCE": 226, "Nota": 2.8, "Logro": "Insuficiente", "Puntaje": 14}</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23209728-0", "7": "FELIPE IGNACIO LARA CAMPOS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.134332</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
-        <v>112</v>
-      </c>
-      <c r="B110" t="n">
-        <v>4</v>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>{"Buenas": 28, "Malas": 11, "Omitidas": 0, "Rend": 71.8, "SIMCE": 303, "Nota": 4.9, "Logro": "Adecuado", "Puntaje": 28}</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23075733-K", "7": "FRANKO JUSTINO CARRASCO BETANCOURT", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.134332</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
-        <v>113</v>
-      </c>
-      <c r="B111" t="n">
-        <v>4</v>
-      </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>{"Buenas": 12, "Malas": 27, "Omitidas": 0, "Rend": 30.8, "SIMCE": 215, "Nota": 2.5, "Logro": "Insuficiente", "Puntaje": 12}</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "22600443-2", "7": "GUSTAVO JES\u00daS GUAJARDO LLONCO\u00d1ANCO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.135332</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
-        <v>114</v>
-      </c>
-      <c r="B112" t="n">
-        <v>4</v>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23206392-0", "7": "HORTENCIA ALEJANDRA ANCAMILLA MILLAL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.135332</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
-        <v>115</v>
-      </c>
-      <c r="B113" t="n">
-        <v>4</v>
-      </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23071865-2", "7": "ISMAEL LUCIANO CALFI\u00d1IR HUENU\u00c1N", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.135332</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
-        <v>116</v>
-      </c>
-      <c r="B114" t="n">
-        <v>4</v>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23284555-4", "7": "JAVIER IGNACIO OLAVARR\u00cdA CUEVAS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.135332</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
-        <v>117</v>
-      </c>
-      <c r="B115" t="n">
-        <v>4</v>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>{"Buenas": 26, "Malas": 13, "Omitidas": 0, "Rend": 66.7, "SIMCE": 292, "Nota": 4.5, "Logro": "Adecuado", "Puntaje": 26}</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "24309656-1", "7": "JEANEN PE\u00d1A", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.135332</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
-        <v>118</v>
-      </c>
-      <c r="B116" t="n">
-        <v>4</v>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>{"Buenas": 27, "Malas": 11, "Omitidas": 1, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23210749-9", "7": "LILIANA IGNACIA MADARIAGA ANCAMILLA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr"/>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.136332</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="n">
-        <v>119</v>
-      </c>
-      <c r="B117" t="n">
-        <v>4</v>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>{"Buenas": 19, "Malas": 20, "Omitidas": 0, "Rend": 48.7, "SIMCE": 254, "Nota": 3.4, "Logro": "Elemental", "Puntaje": 19}</t>
-        </is>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23201622-1", "7": "LUCAS IGNACIO BENJAM\u00cdN ALA\u00d1ANCO BRICE\u00d1O", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.136332</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="n">
-        <v>120</v>
-      </c>
-      <c r="B118" t="n">
-        <v>4</v>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>{"Buenas": 23, "Malas": 16, "Omitidas": 0, "Rend": 59.0, "SIMCE": 276, "Nota": 4.0, "Logro": "Elemental", "Puntaje": 23}</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23169236-3", "7": "MADELEINE INES P\u00c9REZ ESPINOZA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.136332</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="n">
-        <v>121</v>
-      </c>
-      <c r="B119" t="n">
-        <v>4</v>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "22596306-1", "7": "MARTINA ANA\u00cdS G\u00d3MEZ PACHECO", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.136332</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
-        <v>122</v>
-      </c>
-      <c r="B120" t="n">
-        <v>4</v>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>{"Buenas": 21, "Malas": 18, "Omitidas": 0, "Rend": 53.8, "SIMCE": 265, "Nota": 3.7, "Logro": "Elemental", "Puntaje": 21}</t>
-        </is>
-      </c>
-      <c r="D120" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23221210-1", "7": "MARTINA PASCAL LEFIQUEO ANTILEF", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.136332</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
-        <v>123</v>
-      </c>
-      <c r="B121" t="n">
-        <v>4</v>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>{"Buenas": 13, "Malas": 26, "Omitidas": 0, "Rend": 33.3, "SIMCE": 221, "Nota": 2.7, "Logro": "Insuficiente", "Puntaje": 13}</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23207278-4", "7": "MAT\u00cdAS FRANCHESCO \u00c1LAMOS LLEUFUMAN", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.136332</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="n">
-        <v>124</v>
-      </c>
-      <c r="B122" t="n">
-        <v>4</v>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23020358-K", "7": "MOIS\u00c9S ALONSO DUR\u00c1N BERROCAL", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.137331</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="n">
-        <v>125</v>
-      </c>
-      <c r="B123" t="n">
-        <v>4</v>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>{"Buenas": 20, "Malas": 19, "Omitidas": 0, "Rend": 51.3, "SIMCE": 259, "Nota": 3.6, "Logro": "Elemental", "Puntaje": 20}</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "22833690-4", "7": "NAYELI MANQUELIPE BURGOS", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.137331</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
-        <v>126</v>
-      </c>
-      <c r="B124" t="n">
-        <v>4</v>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>{"Buenas": 29, "Malas": 10, "Omitidas": 0, "Rend": 74.4, "SIMCE": 309, "Nota": 5.1, "Logro": "Adecuado", "Puntaje": 29}</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23177773-3", "7": "NEYBER BENJAM\u00cdN CHAND\u00cdA MERA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.137331</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="n">
-        <v>127</v>
-      </c>
-      <c r="B125" t="n">
-        <v>4</v>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>{"Buenas": 16, "Malas": 23, "Omitidas": 0, "Rend": 41.0, "SIMCE": 237, "Nota": 3.1, "Logro": "Insuficiente", "Puntaje": 16}</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23061855-0", "7": "RODRIGO FERNANDO CH\u00c1VEZ MONS\u00c1LVEZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.137331</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="n">
-        <v>128</v>
-      </c>
-      <c r="B126" t="n">
-        <v>4</v>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>{"Buenas": 24, "Malas": 15, "Omitidas": 0, "Rend": 61.5, "SIMCE": 281, "Nota": 4.1, "Logro": "Elemental", "Puntaje": 24}</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23229067-6", "7": "SIGRID NAYARETH BEL\u00c9N BURGOS ESPINOZA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.137834</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="n">
-        <v>129</v>
-      </c>
-      <c r="B127" t="n">
-        <v>4</v>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>{"Buenas": 22, "Malas": 17, "Omitidas": 0, "Rend": 56.4, "SIMCE": 270, "Nota": 3.8, "Logro": "Elemental", "Puntaje": 22}</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23296820-6", "7": "TERECITA DEL NI\u00d1O JES\u00daS CARES MONS\u00c1LVEZ", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>2026-02-13T11:51:15.137834</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
-        <v>130</v>
-      </c>
-      <c r="B128" t="n">
-        <v>4</v>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>{"Buenas": 27, "Malas": 12, "Omitidas": 0, "Rend": 69.2, "SIMCE": 298, "Nota": 4.7, "Logro": "Adecuado", "Puntaje": 27}</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>{"5": "2\u00b0 medio D", "6": "23077160-K", "7": "YOHAN RICARDO PROVOTH ARAVENA", "8": "Lenguaje", "9": "Noviembre", "10": "5", "4": "2025"}</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr"/>
-      <c r="F128" t="inlineStr">
         <is>
           <t>2026-02-13T11:51:15.137834</t>
         </is>

</xml_diff>

<commit_message>
correcciones en gráficos simce
</commit_message>
<xml_diff>
--- a/data/database/metric_data.xlsx
+++ b/data/database/metric_data.xlsx
@@ -480,7 +480,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -528,7 +528,7 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -696,7 +696,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.471479</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -768,7 +768,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.493781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.472982</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.474107</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.474107</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.474107</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.474107</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.474107</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.474107</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1128,7 @@
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.474107</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.474107</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.474107</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.494781</t>
+          <t>2026-03-10T18:08:58.475110</t>
         </is>
       </c>
     </row>
@@ -1224,7 +1224,7 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.475110</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.475110</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1272,7 @@
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.475110</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.475110</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.475110</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1344,7 @@
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.475110</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1368,7 @@
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.475110</t>
         </is>
       </c>
     </row>
@@ -1392,7 +1392,7 @@
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.475110</t>
         </is>
       </c>
     </row>
@@ -1416,7 +1416,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.476109</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.476109</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.476109</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
       <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.476109</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.476612</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1536,7 @@
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.476612</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.495782</t>
+          <t>2026-03-10T18:08:58.476612</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1584,7 @@
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.476612</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.477114</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1632,7 @@
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.477114</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.477114</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1680,7 @@
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.477114</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.477114</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.477114</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1752,7 @@
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478119</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478119</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -1848,7 +1848,7 @@
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1872,7 @@
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -1896,7 +1896,7 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -1920,7 +1920,7 @@
       <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -1944,7 +1944,7 @@
       <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.478627</t>
         </is>
       </c>
     </row>
@@ -2064,7 +2064,7 @@
       <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.480142</t>
         </is>
       </c>
     </row>
@@ -2088,7 +2088,7 @@
       <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.480142</t>
         </is>
       </c>
     </row>
@@ -2112,7 +2112,7 @@
       <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.480142</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.480142</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2160,7 @@
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.480142</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.480142</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.480142</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.480142</t>
         </is>
       </c>
     </row>
@@ -2256,7 +2256,7 @@
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.481145</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2280,7 @@
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.496782</t>
+          <t>2026-03-10T18:08:58.481145</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2304,7 @@
       <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.481145</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2328,7 @@
       <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.481145</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2352,7 @@
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.481145</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.481145</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.481145</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.481145</t>
         </is>
       </c>
     </row>
@@ -2448,7 +2448,7 @@
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.481145</t>
         </is>
       </c>
     </row>
@@ -2472,7 +2472,7 @@
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.482147</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.482147</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.482147</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.482147</t>
         </is>
       </c>
     </row>
@@ -2568,7 +2568,7 @@
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.482147</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2592,7 @@
       <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.482147</t>
         </is>
       </c>
     </row>
@@ -2616,7 +2616,7 @@
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.482147</t>
         </is>
       </c>
     </row>
@@ -2640,7 +2640,7 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.483145</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2664,7 @@
       <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.483145</t>
         </is>
       </c>
     </row>
@@ -2688,7 +2688,7 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.483145</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2712,7 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.498285</t>
+          <t>2026-03-10T18:08:58.483145</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2736,7 @@
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.483145</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.483145</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2784,7 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.483145</t>
         </is>
       </c>
     </row>
@@ -2808,7 +2808,7 @@
       <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.483145</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.483145</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2856,7 @@
       <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.484145</t>
         </is>
       </c>
     </row>
@@ -2880,7 +2880,7 @@
       <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.484145</t>
         </is>
       </c>
     </row>
@@ -2904,7 +2904,7 @@
       <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.484145</t>
         </is>
       </c>
     </row>
@@ -2928,7 +2928,7 @@
       <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.484145</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.484145</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.484145</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3000,7 @@
       <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.484145</t>
         </is>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
       <c r="E108" t="inlineStr"/>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.499288</t>
+          <t>2026-03-10T18:08:58.484145</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3048,7 @@
       <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.613559</t>
+          <t>2026-03-10T18:08:59.496114</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3072,7 @@
       <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.613559</t>
+          <t>2026-03-10T18:08:59.496114</t>
         </is>
       </c>
     </row>
@@ -3096,7 +3096,7 @@
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.613559</t>
+          <t>2026-03-10T18:08:59.496114</t>
         </is>
       </c>
     </row>
@@ -3120,7 +3120,7 @@
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.497150</t>
         </is>
       </c>
     </row>
@@ -3144,7 +3144,7 @@
       <c r="E113" t="inlineStr"/>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.497150</t>
         </is>
       </c>
     </row>
@@ -3168,7 +3168,7 @@
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.497150</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3192,7 @@
       <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.497150</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3216,7 @@
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.497150</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       <c r="E117" t="inlineStr"/>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.497150</t>
         </is>
       </c>
     </row>
@@ -3264,7 +3264,7 @@
       <c r="E118" t="inlineStr"/>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.497150</t>
         </is>
       </c>
     </row>
@@ -3288,7 +3288,7 @@
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.497150</t>
         </is>
       </c>
     </row>
@@ -3312,7 +3312,7 @@
       <c r="E120" t="inlineStr"/>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.498153</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
       <c r="E121" t="inlineStr"/>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.498153</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       <c r="E122" t="inlineStr"/>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.498153</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.498153</t>
         </is>
       </c>
     </row>
@@ -3408,7 +3408,7 @@
       <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.498153</t>
         </is>
       </c>
     </row>
@@ -3432,7 +3432,7 @@
       <c r="E125" t="inlineStr"/>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.498153</t>
         </is>
       </c>
     </row>
@@ -3456,7 +3456,7 @@
       <c r="E126" t="inlineStr"/>
       <c r="F126" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.498153</t>
         </is>
       </c>
     </row>
@@ -3480,7 +3480,7 @@
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.498153</t>
         </is>
       </c>
     </row>
@@ -3504,7 +3504,7 @@
       <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.499154</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
       <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.499154</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.499154</t>
         </is>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
       <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.614559</t>
+          <t>2026-03-10T18:08:59.499154</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3600,7 @@
       <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.499656</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3624,7 @@
       <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.499656</t>
         </is>
       </c>
     </row>
@@ -3648,7 +3648,7 @@
       <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.499656</t>
         </is>
       </c>
     </row>
@@ -3672,7 +3672,7 @@
       <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.499656</t>
         </is>
       </c>
     </row>
@@ -3696,7 +3696,7 @@
       <c r="E136" t="inlineStr"/>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.499656</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3720,7 @@
       <c r="E137" t="inlineStr"/>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.499656</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3744,7 @@
       <c r="E138" t="inlineStr"/>
       <c r="F138" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.499656</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.499656</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3792,7 @@
       <c r="E140" t="inlineStr"/>
       <c r="F140" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.499656</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3816,7 @@
       <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.500659</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3840,7 @@
       <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.500659</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3864,7 @@
       <c r="E143" t="inlineStr"/>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.500659</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3888,7 @@
       <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.500659</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.500659</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
       <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.500659</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3960,7 @@
       <c r="E147" t="inlineStr"/>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.500659</t>
         </is>
       </c>
     </row>
@@ -3984,7 +3984,7 @@
       <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.500659</t>
         </is>
       </c>
     </row>
@@ -4008,7 +4008,7 @@
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.615559</t>
+          <t>2026-03-10T18:08:59.501659</t>
         </is>
       </c>
     </row>
@@ -4032,7 +4032,7 @@
       <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.501659</t>
         </is>
       </c>
     </row>
@@ -4056,7 +4056,7 @@
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.501659</t>
         </is>
       </c>
     </row>
@@ -4080,7 +4080,7 @@
       <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.501659</t>
         </is>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
       <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.501659</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.501659</t>
         </is>
       </c>
     </row>
@@ -4152,7 +4152,7 @@
       <c r="E155" t="inlineStr"/>
       <c r="F155" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.501659</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.501659</t>
         </is>
       </c>
     </row>
@@ -4200,7 +4200,7 @@
       <c r="E157" t="inlineStr"/>
       <c r="F157" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.501659</t>
         </is>
       </c>
     </row>
@@ -4224,7 +4224,7 @@
       <c r="E158" t="inlineStr"/>
       <c r="F158" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.502659</t>
         </is>
       </c>
     </row>
@@ -4248,7 +4248,7 @@
       <c r="E159" t="inlineStr"/>
       <c r="F159" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.502659</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.502659</t>
         </is>
       </c>
     </row>
@@ -4296,7 +4296,7 @@
       <c r="E161" t="inlineStr"/>
       <c r="F161" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.502659</t>
         </is>
       </c>
     </row>
@@ -4320,7 +4320,7 @@
       <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.502659</t>
         </is>
       </c>
     </row>
@@ -4344,7 +4344,7 @@
       <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.502659</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.616560</t>
+          <t>2026-03-10T18:08:59.502659</t>
         </is>
       </c>
     </row>
@@ -4392,7 +4392,7 @@
       <c r="E165" t="inlineStr"/>
       <c r="F165" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.502659</t>
         </is>
       </c>
     </row>
@@ -4416,7 +4416,7 @@
       <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       <c r="E167" t="inlineStr"/>
       <c r="F167" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4464,7 +4464,7 @@
       <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4488,7 +4488,7 @@
       <c r="E169" t="inlineStr"/>
       <c r="F169" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4512,7 @@
       <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4536,7 @@
       <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4560,7 @@
       <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4584,7 +4584,7 @@
       <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4608,7 @@
       <c r="E174" t="inlineStr"/>
       <c r="F174" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4632,7 +4632,7 @@
       <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.503847</t>
         </is>
       </c>
     </row>
@@ -4656,7 +4656,7 @@
       <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.505551</t>
         </is>
       </c>
     </row>
@@ -4680,7 +4680,7 @@
       <c r="E177" t="inlineStr"/>
       <c r="F177" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.505551</t>
         </is>
       </c>
     </row>
@@ -4704,7 +4704,7 @@
       <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.505551</t>
         </is>
       </c>
     </row>
@@ -4728,7 +4728,7 @@
       <c r="E179" t="inlineStr"/>
       <c r="F179" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.505551</t>
         </is>
       </c>
     </row>
@@ -4752,7 +4752,7 @@
       <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.505551</t>
         </is>
       </c>
     </row>
@@ -4776,7 +4776,7 @@
       <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.505551</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4800,7 @@
       <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.505551</t>
         </is>
       </c>
     </row>
@@ -4824,7 +4824,7 @@
       <c r="E183" t="inlineStr"/>
       <c r="F183" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.506557</t>
         </is>
       </c>
     </row>
@@ -4848,7 +4848,7 @@
       <c r="E184" t="inlineStr"/>
       <c r="F184" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.617559</t>
+          <t>2026-03-10T18:08:59.506557</t>
         </is>
       </c>
     </row>
@@ -4872,7 +4872,7 @@
       <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.506557</t>
         </is>
       </c>
     </row>
@@ -4896,7 +4896,7 @@
       <c r="E186" t="inlineStr"/>
       <c r="F186" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.506557</t>
         </is>
       </c>
     </row>
@@ -4920,7 +4920,7 @@
       <c r="E187" t="inlineStr"/>
       <c r="F187" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.507059</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       <c r="E188" t="inlineStr"/>
       <c r="F188" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.507059</t>
         </is>
       </c>
     </row>
@@ -4968,7 +4968,7 @@
       <c r="E189" t="inlineStr"/>
       <c r="F189" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.507059</t>
         </is>
       </c>
     </row>
@@ -4992,7 +4992,7 @@
       <c r="E190" t="inlineStr"/>
       <c r="F190" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.507059</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5016,7 @@
       <c r="E191" t="inlineStr"/>
       <c r="F191" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.507059</t>
         </is>
       </c>
     </row>
@@ -5040,7 +5040,7 @@
       <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.507059</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5064,7 @@
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.507059</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       <c r="E194" t="inlineStr"/>
       <c r="F194" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.507059</t>
         </is>
       </c>
     </row>
@@ -5112,7 +5112,7 @@
       <c r="E195" t="inlineStr"/>
       <c r="F195" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.508064</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.508064</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.508064</t>
         </is>
       </c>
     </row>
@@ -5184,7 +5184,7 @@
       <c r="E198" t="inlineStr"/>
       <c r="F198" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.508568</t>
         </is>
       </c>
     </row>
@@ -5208,7 +5208,7 @@
       <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.508568</t>
         </is>
       </c>
     </row>
@@ -5232,7 +5232,7 @@
       <c r="E200" t="inlineStr"/>
       <c r="F200" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.508568</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5256,7 @@
       <c r="E201" t="inlineStr"/>
       <c r="F201" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.509573</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5280,7 @@
       <c r="E202" t="inlineStr"/>
       <c r="F202" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.509573</t>
         </is>
       </c>
     </row>
@@ -5304,7 +5304,7 @@
       <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.509573</t>
         </is>
       </c>
     </row>
@@ -5328,7 +5328,7 @@
       <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.618673</t>
+          <t>2026-03-10T18:08:59.509573</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5352,7 @@
       <c r="E205" t="inlineStr"/>
       <c r="F205" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.509573</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       <c r="E206" t="inlineStr"/>
       <c r="F206" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.509573</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
       <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.509573</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5424,7 @@
       <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.509573</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       <c r="E209" t="inlineStr"/>
       <c r="F209" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.510577</t>
         </is>
       </c>
     </row>
@@ -5472,7 +5472,7 @@
       <c r="E210" t="inlineStr"/>
       <c r="F210" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.510577</t>
         </is>
       </c>
     </row>
@@ -5496,7 +5496,7 @@
       <c r="E211" t="inlineStr"/>
       <c r="F211" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.510577</t>
         </is>
       </c>
     </row>
@@ -5520,7 +5520,7 @@
       <c r="E212" t="inlineStr"/>
       <c r="F212" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512051</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5544,7 @@
       <c r="E213" t="inlineStr"/>
       <c r="F213" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512051</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5568,7 @@
       <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512051</t>
         </is>
       </c>
     </row>
@@ -5592,7 +5592,7 @@
       <c r="E215" t="inlineStr"/>
       <c r="F215" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512781</t>
         </is>
       </c>
     </row>
@@ -5616,7 +5616,7 @@
       <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512781</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
       <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512781</t>
         </is>
       </c>
     </row>
@@ -5664,7 +5664,7 @@
       <c r="E218" t="inlineStr"/>
       <c r="F218" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512781</t>
         </is>
       </c>
     </row>
@@ -5688,7 +5688,7 @@
       <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512781</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5712,7 @@
       <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512781</t>
         </is>
       </c>
     </row>
@@ -5736,7 +5736,7 @@
       <c r="E221" t="inlineStr"/>
       <c r="F221" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512781</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5760,7 @@
       <c r="E222" t="inlineStr"/>
       <c r="F222" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.512781</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
       <c r="E223" t="inlineStr"/>
       <c r="F223" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.513785</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
       <c r="E224" t="inlineStr"/>
       <c r="F224" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.513785</t>
         </is>
       </c>
     </row>
@@ -5832,7 +5832,7 @@
       <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.619671</t>
+          <t>2026-03-10T18:08:59.513785</t>
         </is>
       </c>
     </row>
@@ -5856,7 +5856,7 @@
       <c r="E226" t="inlineStr"/>
       <c r="F226" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.513785</t>
         </is>
       </c>
     </row>
@@ -5880,7 +5880,7 @@
       <c r="E227" t="inlineStr"/>
       <c r="F227" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.513785</t>
         </is>
       </c>
     </row>
@@ -5904,7 +5904,7 @@
       <c r="E228" t="inlineStr"/>
       <c r="F228" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.513785</t>
         </is>
       </c>
     </row>
@@ -5928,7 +5928,7 @@
       <c r="E229" t="inlineStr"/>
       <c r="F229" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       <c r="E230" t="inlineStr"/>
       <c r="F230" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -5976,7 +5976,7 @@
       <c r="E231" t="inlineStr"/>
       <c r="F231" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -6000,7 +6000,7 @@
       <c r="E232" t="inlineStr"/>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -6024,7 +6024,7 @@
       <c r="E233" t="inlineStr"/>
       <c r="F233" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -6048,7 +6048,7 @@
       <c r="E234" t="inlineStr"/>
       <c r="F234" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6072,7 @@
       <c r="E235" t="inlineStr"/>
       <c r="F235" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -6096,7 +6096,7 @@
       <c r="E236" t="inlineStr"/>
       <c r="F236" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6120,7 @@
       <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -6144,7 +6144,7 @@
       <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.514786</t>
         </is>
       </c>
     </row>
@@ -6168,7 +6168,7 @@
       <c r="E239" t="inlineStr"/>
       <c r="F239" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.516289</t>
         </is>
       </c>
     </row>
@@ -6192,7 +6192,7 @@
       <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.516289</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6216,7 @@
       <c r="E241" t="inlineStr"/>
       <c r="F241" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.516289</t>
         </is>
       </c>
     </row>
@@ -6240,7 +6240,7 @@
       <c r="E242" t="inlineStr"/>
       <c r="F242" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.517294</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6264,7 @@
       <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.517294</t>
         </is>
       </c>
     </row>
@@ -6288,7 +6288,7 @@
       <c r="E244" t="inlineStr"/>
       <c r="F244" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.620671</t>
+          <t>2026-03-10T18:08:59.517798</t>
         </is>
       </c>
     </row>
@@ -6312,7 +6312,7 @@
       <c r="E245" t="inlineStr"/>
       <c r="F245" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.517798</t>
         </is>
       </c>
     </row>
@@ -6336,7 +6336,7 @@
       <c r="E246" t="inlineStr"/>
       <c r="F246" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.517798</t>
         </is>
       </c>
     </row>
@@ -6360,7 +6360,7 @@
       <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.517798</t>
         </is>
       </c>
     </row>
@@ -6384,7 +6384,7 @@
       <c r="E248" t="inlineStr"/>
       <c r="F248" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.518417</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       <c r="E249" t="inlineStr"/>
       <c r="F249" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.518417</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6432,7 @@
       <c r="E250" t="inlineStr"/>
       <c r="F250" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.518417</t>
         </is>
       </c>
     </row>
@@ -6456,7 +6456,7 @@
       <c r="E251" t="inlineStr"/>
       <c r="F251" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.518417</t>
         </is>
       </c>
     </row>
@@ -6480,7 +6480,7 @@
       <c r="E252" t="inlineStr"/>
       <c r="F252" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.518417</t>
         </is>
       </c>
     </row>
@@ -6504,7 +6504,7 @@
       <c r="E253" t="inlineStr"/>
       <c r="F253" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.518417</t>
         </is>
       </c>
     </row>
@@ -6528,7 +6528,7 @@
       <c r="E254" t="inlineStr"/>
       <c r="F254" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.519448</t>
         </is>
       </c>
     </row>
@@ -6552,7 +6552,7 @@
       <c r="E255" t="inlineStr"/>
       <c r="F255" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.519448</t>
         </is>
       </c>
     </row>
@@ -6576,7 +6576,7 @@
       <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.519448</t>
         </is>
       </c>
     </row>
@@ -6600,7 +6600,7 @@
       <c r="E257" t="inlineStr"/>
       <c r="F257" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.519448</t>
         </is>
       </c>
     </row>
@@ -6624,7 +6624,7 @@
       <c r="E258" t="inlineStr"/>
       <c r="F258" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.519448</t>
         </is>
       </c>
     </row>
@@ -6648,7 +6648,7 @@
       <c r="E259" t="inlineStr"/>
       <c r="F259" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.520452</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6672,7 @@
       <c r="E260" t="inlineStr"/>
       <c r="F260" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.520452</t>
         </is>
       </c>
     </row>
@@ -6696,7 +6696,7 @@
       <c r="E261" t="inlineStr"/>
       <c r="F261" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.520452</t>
         </is>
       </c>
     </row>
@@ -6720,7 +6720,7 @@
       <c r="E262" t="inlineStr"/>
       <c r="F262" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.520452</t>
         </is>
       </c>
     </row>
@@ -6744,7 +6744,7 @@
       <c r="E263" t="inlineStr"/>
       <c r="F263" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.521453</t>
         </is>
       </c>
     </row>
@@ -6768,7 +6768,7 @@
       <c r="E264" t="inlineStr"/>
       <c r="F264" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.621671</t>
+          <t>2026-03-10T18:08:59.521453</t>
         </is>
       </c>
     </row>
@@ -6792,7 +6792,7 @@
       <c r="E265" t="inlineStr"/>
       <c r="F265" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.622671</t>
+          <t>2026-03-10T18:08:59.521453</t>
         </is>
       </c>
     </row>
@@ -6816,7 +6816,7 @@
       <c r="E266" t="inlineStr"/>
       <c r="F266" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.622671</t>
+          <t>2026-03-10T18:08:59.521453</t>
         </is>
       </c>
     </row>
@@ -6840,7 +6840,7 @@
       <c r="E267" t="inlineStr"/>
       <c r="F267" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.622671</t>
+          <t>2026-03-10T18:08:59.521453</t>
         </is>
       </c>
     </row>
@@ -6864,7 +6864,7 @@
       <c r="E268" t="inlineStr"/>
       <c r="F268" t="inlineStr">
         <is>
-          <t>2026-03-10T16:13:02.622671</t>
+          <t>2026-03-10T18:08:59.522452</t>
         </is>
       </c>
     </row>

</xml_diff>